<commit_message>
possible replacement for 2.2uH inductor
excel sheet changes
</commit_message>
<xml_diff>
--- a/Spaceport/PCBs/ARCH-Mega/BOM/ARCH-Mega_BOM.xlsx
+++ b/Spaceport/PCBs/ARCH-Mega/BOM/ARCH-Mega_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\malav_16\College\terrapin_rocket\github\SRAD_Avionics_1\SRAD-Avionics\Spaceport\PCBs\ARCH-Mega\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95025486-0E3D-481A-BE63-03CB95795A57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D577AAF-582E-48DC-898F-87DAB8C41FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{BFC3F118-C025-4DFF-9FE5-C20B848F3DC7}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="201">
   <si>
     <t>Reference</t>
   </si>
@@ -617,6 +617,12 @@
   </si>
   <si>
     <t>https://www.digikey.com/en/products/detail/arlitech-electronic-corp/AMPI0640ED2R2MT/20415872?s=N4IgTCBcDaIIIFkAKBJADANgCxoKIBEwAlMBAFRAF0BfIA</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/w%C3%BCrth-elektronik/744311220/1638556</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Possible Replacement </t>
   </si>
 </sst>
 </file>
@@ -1529,7 +1535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EDC2ABD5-0CB0-4FAD-9A39-002E1327DB07}">
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="57.5703125" customWidth="1"/>
@@ -1541,9 +1547,10 @@
     <col min="7" max="7" width="17.42578125" customWidth="1"/>
     <col min="8" max="8" width="19.85546875" customWidth="1"/>
     <col min="9" max="9" width="29.140625" customWidth="1"/>
+    <col min="10" max="10" width="43.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1571,8 +1578,11 @@
       <c r="I1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1601,7 +1611,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1618,7 +1628,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1635,7 +1645,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -1652,7 +1662,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -1669,7 +1679,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1686,7 +1696,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1703,7 +1713,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1720,7 +1730,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1737,7 +1747,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -1754,7 +1764,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -1771,7 +1781,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1788,7 +1798,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -1814,7 +1824,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -1831,7 +1841,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>38</v>
       </c>
@@ -1857,7 +1867,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -1883,7 +1893,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>44</v>
       </c>
@@ -1912,7 +1922,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>48</v>
       </c>
@@ -1938,7 +1948,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -1964,7 +1974,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>54</v>
       </c>
@@ -1990,7 +2000,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>57</v>
       </c>
@@ -2016,7 +2026,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>60</v>
       </c>
@@ -2039,7 +2049,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>63</v>
       </c>
@@ -2061,8 +2071,11 @@
       <c r="I24" s="1" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -2088,7 +2101,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -2117,7 +2130,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>73</v>
       </c>
@@ -2146,7 +2159,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>75</v>
       </c>
@@ -2175,7 +2188,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>78</v>
       </c>
@@ -2192,7 +2205,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -2209,7 +2222,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>83</v>
       </c>
@@ -2226,7 +2239,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>85</v>
       </c>
@@ -2812,7 +2825,7 @@
       <formula>NOT(ISERROR(SEARCH("In Stock",G61)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2 H14 H16:H28 H50:H57 F57:G57 G2:G56">
+  <conditionalFormatting sqref="H2 G2:G56 H14 H16:H28 H50:H57 F57:G57">
     <cfRule type="containsText" dxfId="1" priority="5" operator="containsText" text="Out of Stock">
       <formula>NOT(ISERROR(SEARCH("Out of Stock",F2)))</formula>
     </cfRule>
@@ -2857,6 +2870,7 @@
     <hyperlink ref="I2" r:id="rId23" xr:uid="{C92553D5-957D-4E64-9369-0B5BB0A2EB40}"/>
     <hyperlink ref="I14" r:id="rId24" xr:uid="{C236FADA-DCE4-471C-A728-829F6B2C2CFB}"/>
     <hyperlink ref="I24" r:id="rId25" xr:uid="{8B948C4F-FCC5-4A54-80F6-6F1A1170409C}"/>
+    <hyperlink ref="J24" r:id="rId26" xr:uid="{3AA44EA1-C6BA-4D1D-9759-3BD8A205943A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>